<commit_message>
Used vlooup and Index - Match function
</commit_message>
<xml_diff>
--- a/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
+++ b/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT_VEDANT\EXCEL\lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11A9619C-0A07-40BB-945A-B9E0960AD859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B943BFF-F28C-4623-8090-877DDA09E15F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DMartDataset" sheetId="1" r:id="rId1"/>
@@ -19,11 +19,11 @@
     <sheet name="if_formula" sheetId="5" r:id="rId4"/>
     <sheet name="custome_list" sheetId="4" r:id="rId5"/>
     <sheet name="Sheet1" sheetId="6" r:id="rId6"/>
-    <sheet name="Sheet2" sheetId="7" r:id="rId7"/>
-    <sheet name="Sheet4" sheetId="8" r:id="rId8"/>
+    <sheet name="Sheet4" sheetId="8" r:id="rId7"/>
+    <sheet name="vlookup" sheetId="7" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Sheet4!$B$2:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Sheet4!$B$2:$B$9</definedName>
     <definedName name="Category">DMart_Sales_data[Category]</definedName>
     <definedName name="customer_type">DMart_Sales_data[customer_type]</definedName>
     <definedName name="Discount">DMart_Sales_data[discount]</definedName>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4208" uniqueCount="690">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4217" uniqueCount="696">
   <si>
     <t>Region</t>
   </si>
@@ -2147,6 +2147,24 @@
   </si>
   <si>
     <t>Total Sales (using subtotal)</t>
+  </si>
+  <si>
+    <t>Emp_ID</t>
+  </si>
+  <si>
+    <t>EmployeeID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MATCH </t>
+  </si>
+  <si>
+    <t>POSITION</t>
+  </si>
+  <si>
+    <t>Using Vlookup</t>
+  </si>
+  <si>
+    <t>Using INDEX MATCH</t>
   </si>
 </sst>
 </file>
@@ -2616,12 +2634,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2630,7 +2648,7 @@
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3447,7 +3465,7 @@
     <col min="18" max="18" width="61.5546875" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="13" customWidth="1"/>
     <col min="20" max="20" width="8.6640625" customWidth="1"/>
-    <col min="21" max="21" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11" bestFit="1" customWidth="1"/>
     <col min="22" max="25" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -49606,77 +49624,6 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A9FE236-3953-4E80-94B6-5B72F4EC6BD0}">
-  <dimension ref="A1:A12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" s="26" t="s">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" s="26" t="s">
-        <v>583</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="26" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" s="26" t="s">
-        <v>585</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" s="26" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" s="26" t="s">
-        <v>590</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" s="26" t="s">
-        <v>591</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" s="26" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" s="26" t="s">
-        <v>592</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" s="26" t="s">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" s="26" t="s">
-        <v>594</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="14" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{607087B3-0129-4C63-A08A-77F360FD7DD5}">
   <dimension ref="B1:J11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -49695,10 +49642,10 @@
       <c r="B3" s="63">
         <v>120</v>
       </c>
-      <c r="E3" s="65" t="s">
+      <c r="E3" s="60" t="s">
         <v>685</v>
       </c>
-      <c r="I3" s="65" t="s">
+      <c r="I3" s="60" t="s">
         <v>687</v>
       </c>
     </row>
@@ -49711,14 +49658,14 @@
       <c r="B5" s="63">
         <v>150</v>
       </c>
-      <c r="D5" s="65" t="s">
+      <c r="D5" s="60" t="s">
         <v>684</v>
       </c>
       <c r="E5">
         <f>SUBTOTAL(9,B3:B9)</f>
         <v>469</v>
       </c>
-      <c r="I5" s="65" t="s">
+      <c r="I5" s="60" t="s">
         <v>686</v>
       </c>
       <c r="J5">
@@ -49751,14 +49698,219 @@
       <c r="D9" s="61"/>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B10" s="65"/>
-      <c r="C10" s="65"/>
+      <c r="B10" s="60"/>
+      <c r="C10" s="60"/>
     </row>
     <row r="11" spans="2:10" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C11" s="65"/>
+      <c r="C11" s="60"/>
     </row>
   </sheetData>
   <autoFilter ref="B2:B9" xr:uid="{607087B3-0129-4C63-A08A-77F360FD7DD5}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A9FE236-3953-4E80-94B6-5B72F4EC6BD0}">
+  <dimension ref="A2:G15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="32" t="s">
+        <v>690</v>
+      </c>
+      <c r="B2" s="32" t="s">
+        <v>597</v>
+      </c>
+      <c r="C2" s="32" t="s">
+        <v>576</v>
+      </c>
+      <c r="D2" s="32" t="s">
+        <v>621</v>
+      </c>
+      <c r="E2" s="32" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="33">
+        <v>1001</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>548</v>
+      </c>
+      <c r="C3" s="34">
+        <v>70000</v>
+      </c>
+      <c r="D3" s="36">
+        <f>IF(C3&gt;=$G$13,15%,IF(C3&gt;=$G$14,10%,IF(C3&gt;=$G$15,5%,0%)))</f>
+        <v>0.15</v>
+      </c>
+      <c r="E3" s="34">
+        <f>C3*D3</f>
+        <v>10500</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="33">
+        <v>1002</v>
+      </c>
+      <c r="B4" s="33" t="s">
+        <v>579</v>
+      </c>
+      <c r="C4" s="34">
+        <v>50000</v>
+      </c>
+      <c r="D4" s="36">
+        <f>IF(C4&gt;=$G$13,15%,IF(C4&gt;=$G$14,10%,IF(C4&gt;=$G$15,5%,0%)))</f>
+        <v>0.15</v>
+      </c>
+      <c r="E4" s="34">
+        <f>C4*D4</f>
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="33">
+        <v>1003</v>
+      </c>
+      <c r="B5" s="33" t="s">
+        <v>602</v>
+      </c>
+      <c r="C5" s="34">
+        <v>45000</v>
+      </c>
+      <c r="D5" s="36">
+        <f>IF(C5&gt;=$G$13,15%,IF(C5&gt;=$G$14,10%,IF(C5&gt;=$G$15,5%,0%)))</f>
+        <v>0.15</v>
+      </c>
+      <c r="E5" s="34">
+        <f>C5*D5</f>
+        <v>6750</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="35">
+        <v>1004</v>
+      </c>
+      <c r="B6" s="35" t="s">
+        <v>546</v>
+      </c>
+      <c r="C6" s="34">
+        <v>75000</v>
+      </c>
+      <c r="D6" s="36">
+        <f>IF(C6&gt;=$G$13,15%,IF(C6&gt;=$G$14,10%,IF(C6&gt;=$G$15,5%,0%)))</f>
+        <v>0.15</v>
+      </c>
+      <c r="E6" s="34">
+        <f>C6*D6</f>
+        <v>11250</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="35">
+        <v>1005</v>
+      </c>
+      <c r="B7" s="35" t="s">
+        <v>620</v>
+      </c>
+      <c r="C7" s="34">
+        <v>55000</v>
+      </c>
+      <c r="D7" s="36">
+        <f>IF(C7&gt;=$G$13,15%,IF(C7&gt;=$G$14,10%,IF(C7&gt;=$G$15,5%,0%)))</f>
+        <v>0.15</v>
+      </c>
+      <c r="E7" s="34">
+        <f>C7*D7</f>
+        <v>8250</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B9" s="27" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B10" s="65" t="s">
+        <v>691</v>
+      </c>
+      <c r="C10" s="65" t="s">
+        <v>576</v>
+      </c>
+      <c r="D10" s="65" t="s">
+        <v>624</v>
+      </c>
+      <c r="F10" s="65" t="s">
+        <v>692</v>
+      </c>
+      <c r="G10" s="65" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B11">
+        <v>1003</v>
+      </c>
+      <c r="C11">
+        <f>VLOOKUP(B11,A3:E7,MATCH(C2,A2:E2,0),FALSE)</f>
+        <v>45000</v>
+      </c>
+      <c r="D11">
+        <f>VLOOKUP(B11,A3:E7,MATCH(E2,A2:E2,0),FALSE)</f>
+        <v>6750</v>
+      </c>
+      <c r="F11" t="s">
+        <v>602</v>
+      </c>
+      <c r="G11">
+        <f>MATCH(F11,B2:B7,0)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B13" s="27" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B14" s="65" t="s">
+        <v>691</v>
+      </c>
+      <c r="C14" s="65" t="s">
+        <v>576</v>
+      </c>
+      <c r="D14" s="65" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B15">
+        <v>1005</v>
+      </c>
+      <c r="C15">
+        <f>INDEX(C3:C7,MATCH(B15,A3:A7,0))</f>
+        <v>55000</v>
+      </c>
+      <c r="D15">
+        <f>INDEX(E3:E7,MATCH(B15,A3:A7,0))</f>
+        <v>8250</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="14" type="noConversion"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B11 B15" xr:uid="{4A439758-2AD6-4796-909D-A3AB5C5BB3DD}">
+      <formula1>$A$3:$A$7</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Done Data Validation and vlookup
</commit_message>
<xml_diff>
--- a/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
+++ b/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
@@ -8,25 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT_VEDANT\EXCEL\lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B943BFF-F28C-4623-8090-877DDA09E15F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A62F25B-4651-425C-8403-E5C48B6B02FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="659" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DMartDataset" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet5" sheetId="9" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="SUMIF" sheetId="9" r:id="rId2"/>
+    <sheet name="TEXT TO COLUMN" sheetId="3" r:id="rId3"/>
     <sheet name="if_formula" sheetId="5" r:id="rId4"/>
     <sheet name="custome_list" sheetId="4" r:id="rId5"/>
-    <sheet name="Sheet1" sheetId="6" r:id="rId6"/>
-    <sheet name="Sheet4" sheetId="8" r:id="rId7"/>
+    <sheet name="nested if" sheetId="6" r:id="rId6"/>
+    <sheet name="subtotal" sheetId="8" r:id="rId7"/>
     <sheet name="vlookup" sheetId="7" r:id="rId8"/>
+    <sheet name="hlookup" sheetId="10" r:id="rId9"/>
+    <sheet name="Hlookup1" sheetId="11" r:id="rId10"/>
+    <sheet name="INDIRECT" sheetId="12" r:id="rId11"/>
+    <sheet name="Data Validation" sheetId="13" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Sheet4!$B$2:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">subtotal!$B$2:$B$9</definedName>
+    <definedName name="Apples">INDIRECT!$B$2:$B$6</definedName>
+    <definedName name="Bananas">INDIRECT!$C$2:$C$6</definedName>
     <definedName name="Category">DMart_Sales_data[Category]</definedName>
     <definedName name="customer_type">DMart_Sales_data[customer_type]</definedName>
     <definedName name="Discount">DMart_Sales_data[discount]</definedName>
+    <definedName name="Lemons">INDIRECT!$D$2:$D$6</definedName>
     <definedName name="oder_date">DMart_Sales_data[order_date]</definedName>
     <definedName name="Oders">DMart_Sales_data[Oder_ID]</definedName>
     <definedName name="payment_mode">DMart_Sales_data[payment_mode]</definedName>
@@ -48,7 +55,7 @@
       </xcalcf:calcFeatures>
     </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="gT5L9Uh5Mkce+NjaHPxVAbIJlDW9RbqkjfO6mNdsl18="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId13" roundtripDataChecksum="gT5L9Uh5Mkce+NjaHPxVAbIJlDW9RbqkjfO6mNdsl18="/>
     </ext>
   </extLst>
 </workbook>
@@ -77,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4217" uniqueCount="696">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4279" uniqueCount="727">
   <si>
     <t>Region</t>
   </si>
@@ -1786,18 +1793,6 @@
     <t>Contact-No</t>
   </si>
   <si>
-    <t>91-8967598967</t>
-  </si>
-  <si>
-    <t>91-9878586967</t>
-  </si>
-  <si>
-    <t>91-9089788767</t>
-  </si>
-  <si>
-    <t>91-8978877890</t>
-  </si>
-  <si>
     <t>10 digt</t>
   </si>
   <si>
@@ -2165,22 +2160,135 @@
   </si>
   <si>
     <t>Using INDEX MATCH</t>
+  </si>
+  <si>
+    <t>Bonus amount</t>
+  </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>Feb</t>
+  </si>
+  <si>
+    <t>Mar</t>
+  </si>
+  <si>
+    <t>Apr</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>Travel</t>
+  </si>
+  <si>
+    <t>Profit</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">using VLOOKUP </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>B2</t>
+  </si>
+  <si>
+    <t>R5C</t>
+  </si>
+  <si>
+    <t>Bananas</t>
+  </si>
+  <si>
+    <t>Lemons</t>
+  </si>
+  <si>
+    <t>Amit</t>
+  </si>
+  <si>
+    <t>Neha</t>
+  </si>
+  <si>
+    <t>Ketan</t>
+  </si>
+  <si>
+    <t>Sunil</t>
+  </si>
+  <si>
+    <t>Pooja</t>
+  </si>
+  <si>
+    <t>Fruit</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Averages</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>Min</t>
+  </si>
+  <si>
+    <t>Age</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>MIN</t>
+  </si>
+  <si>
+    <t>MAX</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>greter than</t>
+  </si>
+  <si>
+    <t>less than</t>
+  </si>
+  <si>
+    <t>OTP</t>
+  </si>
+  <si>
+    <t>KHIH</t>
+  </si>
+  <si>
+    <t>OrderID</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="[$-14009]dd\-mm\-yyyy;@"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2554,101 +2662,112 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="12" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="13" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="6" fontId="17" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="6" fontId="18" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3471,13 +3590,13 @@
   <sheetData>
     <row r="1" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="20" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="B1" s="21" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>574</v>
+        <v>570</v>
       </c>
       <c r="D1" s="21" t="s">
         <v>1</v>
@@ -3486,7 +3605,7 @@
         <v>2</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>629</v>
+        <v>625</v>
       </c>
       <c r="G1" s="22" t="s">
         <v>3</v>
@@ -3516,7 +3635,7 @@
         <v>10</v>
       </c>
       <c r="P1" s="43" t="s">
-        <v>632</v>
+        <v>628</v>
       </c>
       <c r="Q1" s="25"/>
       <c r="R1" s="1"/>
@@ -3584,7 +3703,7 @@
       <c r="Q2" s="25"/>
       <c r="R2" s="1"/>
       <c r="S2" s="1" t="s">
-        <v>631</v>
+        <v>627</v>
       </c>
       <c r="T2" s="1"/>
       <c r="U2" s="1"/>
@@ -3600,10 +3719,10 @@
         <v>17</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>18</v>
@@ -3649,7 +3768,7 @@
       <c r="Q3" s="25"/>
       <c r="R3" s="1"/>
       <c r="S3" s="1" t="s">
-        <v>630</v>
+        <v>626</v>
       </c>
       <c r="T3" s="1"/>
       <c r="U3" s="1"/>
@@ -3839,7 +3958,7 @@
       </c>
       <c r="Q6" s="25"/>
       <c r="R6" s="44" t="s">
-        <v>634</v>
+        <v>630</v>
       </c>
       <c r="S6" s="45">
         <f>SUMIF(DMart_Sales_data[payment_mode],"=UPI",DMart_Sales_data[sales])</f>
@@ -3859,10 +3978,10 @@
         <v>32</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>33</v>
@@ -3906,7 +4025,7 @@
         <v>Yes</v>
       </c>
       <c r="R7" s="44" t="s">
-        <v>635</v>
+        <v>631</v>
       </c>
       <c r="S7" s="45">
         <f>SUMIF(DMart_Sales_data[payment_mode],"=Card",DMart_Sales_data[sales])</f>
@@ -3973,7 +4092,7 @@
         <v>No</v>
       </c>
       <c r="R8" s="44" t="s">
-        <v>636</v>
+        <v>632</v>
       </c>
       <c r="S8" s="45">
         <f>SUMIF(DMart_Sales_data[payment_mode],"=Cash",DMart_Sales_data[sales])</f>
@@ -4103,7 +4222,7 @@
       </c>
       <c r="Q10" s="1"/>
       <c r="R10" s="50" t="s">
-        <v>651</v>
+        <v>647</v>
       </c>
       <c r="S10" s="27">
         <f>SUMIFS(DMart_Sales_data[sales],DMart_Sales_data[Category],"=Clothing",DMart_Sales_data[Updated_Result],"=East")</f>
@@ -4123,10 +4242,10 @@
         <v>41</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D11" s="10" t="s">
         <v>33</v>
@@ -4234,7 +4353,7 @@
       </c>
       <c r="Q12" s="1"/>
       <c r="R12" s="50" t="s">
-        <v>652</v>
+        <v>648</v>
       </c>
       <c r="S12" s="50">
         <f>SUMIFS(DMart_Sales_data[sales],DMart_Sales_data[Updated_Result],"North",DMart_Sales_data[Category],"Electronics",DMart_Sales_data[discount],"&gt;40%")</f>
@@ -4378,10 +4497,10 @@
         <v>46</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>13</v>
@@ -4426,7 +4545,7 @@
       </c>
       <c r="Q15" s="1"/>
       <c r="R15" s="25" t="s">
-        <v>655</v>
+        <v>651</v>
       </c>
       <c r="S15" s="19"/>
       <c r="T15" s="19"/>
@@ -4491,7 +4610,7 @@
       </c>
       <c r="Q16" s="1"/>
       <c r="R16" s="50" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
       <c r="S16" s="50">
         <f>COUNT(Sales)</f>
@@ -4559,7 +4678,7 @@
       </c>
       <c r="Q17" s="1"/>
       <c r="R17" s="51" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="S17" s="52">
         <f>COUNTIF(DMart_Sales_data[payment_mode],"=UPI")</f>
@@ -4627,7 +4746,7 @@
       </c>
       <c r="Q18" s="1"/>
       <c r="R18" s="51" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="S18" s="52">
         <f>COUNTIF(DMart_Sales_data[payment_mode],"=Card")</f>
@@ -4647,10 +4766,10 @@
         <v>52</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D19" s="10" t="s">
         <v>13</v>
@@ -4695,7 +4814,7 @@
       </c>
       <c r="Q19" s="1"/>
       <c r="R19" s="51" t="s">
-        <v>658</v>
+        <v>654</v>
       </c>
       <c r="S19" s="52">
         <f>COUNTIF(DMart_Sales_data[payment_mode],"=Cash")</f>
@@ -4885,7 +5004,7 @@
       </c>
       <c r="Q22" s="1"/>
       <c r="R22" s="51" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
       <c r="S22" s="53" cm="1">
         <f t="array" ref="S22">COUNTIF(Sales,"&gt;4000")</f>
@@ -4905,10 +5024,10 @@
         <v>58</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D23" s="10" t="s">
         <v>33</v>
@@ -4953,7 +5072,7 @@
       </c>
       <c r="Q23" s="1"/>
       <c r="R23" s="51" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="S23" s="53" cm="1">
         <f t="array" ref="S23">COUNTIFS(Sales,"&gt;4000",DMart_Sales_data[Updated_Result],"=East")</f>
@@ -5021,7 +5140,7 @@
       </c>
       <c r="Q24" s="1"/>
       <c r="R24" s="51" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
       <c r="S24" s="53" cm="1">
         <f t="array" ref="S24">COUNTIFS(Sales,"&gt;4000",DMart_Sales_data[Updated_Result],"West")</f>
@@ -5089,7 +5208,7 @@
       </c>
       <c r="Q25" s="1"/>
       <c r="R25" s="51" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
       <c r="S25" s="53" cm="1">
         <f t="array" ref="S25">COUNTIFS(Sales,"&gt;4000",DMart_Sales_data[Updated_Result],"North")</f>
@@ -5157,7 +5276,7 @@
       </c>
       <c r="Q26" s="1"/>
       <c r="R26" s="51" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="S26" s="53" cm="1">
         <f t="array" ref="S26">COUNTIFS(Sales,"&gt;4000",DMart_Sales_data[Updated_Result],"South")</f>
@@ -5177,10 +5296,10 @@
         <v>63</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D27" s="10" t="s">
         <v>33</v>
@@ -5286,7 +5405,7 @@
       </c>
       <c r="Q28" s="1"/>
       <c r="R28" s="54" t="s">
-        <v>664</v>
+        <v>660</v>
       </c>
       <c r="S28" cm="1">
         <f t="array" ref="S28">COUNTIFS(customer_type,"=Member",payment_mode,"=UPI")+COUNTIFS(customer_type,"=Member",payment_mode,"=Card")</f>
@@ -5417,7 +5536,7 @@
       </c>
       <c r="Q30" s="1"/>
       <c r="R30" s="56" t="s">
-        <v>665</v>
+        <v>661</v>
       </c>
       <c r="S30" s="53" cm="1">
         <f t="array" ref="S30">SUMIF(Regions,"North",Sales)</f>
@@ -5437,10 +5556,10 @@
         <v>69</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D31" s="10" t="s">
         <v>13</v>
@@ -5485,7 +5604,7 @@
       </c>
       <c r="Q31" s="1"/>
       <c r="R31" s="56" t="s">
-        <v>666</v>
+        <v>662</v>
       </c>
       <c r="S31" s="53" cm="1">
         <f t="array" ref="S31">SUMIF(Regions,"South",Sales)</f>
@@ -5553,7 +5672,7 @@
       </c>
       <c r="Q32" s="1"/>
       <c r="R32" s="56" t="s">
-        <v>667</v>
+        <v>663</v>
       </c>
       <c r="S32" s="53" cm="1">
         <f t="array" ref="S32">SUMIF(Regions,"East",Sales)</f>
@@ -5621,7 +5740,7 @@
       </c>
       <c r="Q33" s="1"/>
       <c r="R33" s="56" t="s">
-        <v>668</v>
+        <v>664</v>
       </c>
       <c r="S33" s="53" cm="1">
         <f t="array" ref="S33">SUMIF(Regions,"West",Sales)</f>
@@ -5704,10 +5823,10 @@
         <v>73</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D35" s="10" t="s">
         <v>13</v>
@@ -5752,7 +5871,7 @@
       </c>
       <c r="Q35" s="1"/>
       <c r="R35" s="55" t="s">
-        <v>669</v>
+        <v>665</v>
       </c>
       <c r="S35" s="1"/>
       <c r="T35" s="1"/>
@@ -5880,7 +5999,7 @@
       </c>
       <c r="Q37" s="1"/>
       <c r="R37" s="56" t="s">
-        <v>670</v>
+        <v>666</v>
       </c>
       <c r="S37" s="53">
         <f>COUNTIF(DMart_Sales_data[Updated_Result],"East")</f>
@@ -5948,7 +6067,7 @@
       </c>
       <c r="Q38" s="1"/>
       <c r="R38" s="56" t="s">
-        <v>671</v>
+        <v>667</v>
       </c>
       <c r="S38" s="53">
         <f>COUNTIF(DMart_Sales_data[Updated_Result],"West")</f>
@@ -5968,10 +6087,10 @@
         <v>77</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D39" s="10" t="s">
         <v>33</v>
@@ -6016,7 +6135,7 @@
       </c>
       <c r="Q39" s="1"/>
       <c r="R39" s="56" t="s">
-        <v>672</v>
+        <v>668</v>
       </c>
       <c r="S39" s="53">
         <f>COUNTIF(DMart_Sales_data[Updated_Result],"North")</f>
@@ -6084,7 +6203,7 @@
       </c>
       <c r="Q40" s="1"/>
       <c r="R40" s="56" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="S40" s="53">
         <f>COUNTIF(DMart_Sales_data[Updated_Result],"South")</f>
@@ -6230,10 +6349,10 @@
         <v>82</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D43" s="10" t="s">
         <v>36</v>
@@ -6278,7 +6397,7 @@
       </c>
       <c r="Q43" s="1"/>
       <c r="R43" s="55" t="s">
-        <v>674</v>
+        <v>670</v>
       </c>
       <c r="S43" s="1" cm="1">
         <f t="array" ref="S43">SUMIF(oder_date,"&lt;01/01/2024",Sales)</f>
@@ -6346,7 +6465,7 @@
       </c>
       <c r="Q44" s="1"/>
       <c r="R44" s="55" t="s">
-        <v>675</v>
+        <v>671</v>
       </c>
       <c r="S44" s="1" cm="1">
         <f t="array" ref="S44">SUMIFS(Sales,oder_date,"&gt;=2024/07/01",oder_date,"&lt;=2024/12/31")</f>
@@ -6495,10 +6614,10 @@
         <v>86</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D47" s="10" t="s">
         <v>24</v>
@@ -6543,7 +6662,7 @@
       </c>
       <c r="Q47" s="1"/>
       <c r="R47" s="57" t="s">
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="S47" s="1"/>
       <c r="T47" s="1"/>
@@ -6670,9 +6789,15 @@
         <v>No</v>
       </c>
       <c r="Q49" s="1"/>
-      <c r="R49" s="1"/>
-      <c r="S49" s="1"/>
-      <c r="T49" s="1"/>
+      <c r="R49" s="56" t="s">
+        <v>726</v>
+      </c>
+      <c r="S49" s="56" t="s">
+        <v>572</v>
+      </c>
+      <c r="T49" s="56" t="s">
+        <v>9</v>
+      </c>
       <c r="U49" s="1"/>
       <c r="V49" s="1"/>
       <c r="W49" s="1"/>
@@ -6733,6 +6858,13 @@
         <v>No</v>
       </c>
       <c r="Q50" s="1"/>
+      <c r="R50" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="S50" s="34">
+        <f>VLOOKUP(R50,DMart_Sales_data[],MATCH(DMart_Sales_data[[#Headers],[sales]],DMart_Sales_data[#Headers],0),FALSE)</f>
+        <v>3802.97</v>
+      </c>
       <c r="U50" s="1"/>
       <c r="V50" s="1"/>
       <c r="W50" s="1"/>
@@ -6746,10 +6878,10 @@
         <v>90</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D51" s="10" t="s">
         <v>33</v>
@@ -6995,10 +7127,10 @@
         <v>95</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D55" s="10" t="s">
         <v>18</v>
@@ -7247,10 +7379,10 @@
         <v>100</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D59" s="10" t="s">
         <v>18</v>
@@ -7499,10 +7631,10 @@
         <v>104</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D63" s="10" t="s">
         <v>13</v>
@@ -7751,10 +7883,10 @@
         <v>108</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D67" s="10" t="s">
         <v>33</v>
@@ -8003,10 +8135,10 @@
         <v>112</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D71" s="10" t="s">
         <v>33</v>
@@ -8255,10 +8387,10 @@
         <v>116</v>
       </c>
       <c r="B75" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D75" s="10" t="s">
         <v>24</v>
@@ -8507,10 +8639,10 @@
         <v>120</v>
       </c>
       <c r="B79" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D79" s="10" t="s">
         <v>18</v>
@@ -8759,10 +8891,10 @@
         <v>124</v>
       </c>
       <c r="B83" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D83" s="10" t="s">
         <v>13</v>
@@ -9011,10 +9143,10 @@
         <v>128</v>
       </c>
       <c r="B87" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D87" s="10" t="s">
         <v>36</v>
@@ -9263,10 +9395,10 @@
         <v>132</v>
       </c>
       <c r="B91" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D91" s="10" t="s">
         <v>33</v>
@@ -9515,10 +9647,10 @@
         <v>136</v>
       </c>
       <c r="B95" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D95" s="10" t="s">
         <v>24</v>
@@ -9767,10 +9899,10 @@
         <v>140</v>
       </c>
       <c r="B99" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D99" s="10" t="s">
         <v>33</v>
@@ -10019,10 +10151,10 @@
         <v>144</v>
       </c>
       <c r="B103" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D103" s="10" t="s">
         <v>33</v>
@@ -10271,10 +10403,10 @@
         <v>148</v>
       </c>
       <c r="B107" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D107" s="10" t="s">
         <v>33</v>
@@ -10517,10 +10649,10 @@
         <v>152</v>
       </c>
       <c r="B111" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C111" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D111" s="10" t="s">
         <v>36</v>
@@ -10769,10 +10901,10 @@
         <v>156</v>
       </c>
       <c r="B115" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C115" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D115" s="10" t="s">
         <v>36</v>
@@ -11021,10 +11153,10 @@
         <v>160</v>
       </c>
       <c r="B119" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D119" s="10" t="s">
         <v>33</v>
@@ -11273,10 +11405,10 @@
         <v>164</v>
       </c>
       <c r="B123" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C123" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D123" s="10" t="s">
         <v>33</v>
@@ -11525,10 +11657,10 @@
         <v>168</v>
       </c>
       <c r="B127" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C127" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D127" s="10" t="s">
         <v>36</v>
@@ -11777,10 +11909,10 @@
         <v>172</v>
       </c>
       <c r="B131" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C131" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D131" s="10" t="s">
         <v>18</v>
@@ -12029,10 +12161,10 @@
         <v>176</v>
       </c>
       <c r="B135" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C135" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D135" s="10" t="s">
         <v>36</v>
@@ -12281,10 +12413,10 @@
         <v>180</v>
       </c>
       <c r="B139" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C139" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D139" s="10" t="s">
         <v>24</v>
@@ -12533,10 +12665,10 @@
         <v>184</v>
       </c>
       <c r="B143" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C143" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D143" s="10" t="s">
         <v>13</v>
@@ -12785,10 +12917,10 @@
         <v>188</v>
       </c>
       <c r="B147" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C147" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D147" s="10" t="s">
         <v>33</v>
@@ -13037,10 +13169,10 @@
         <v>192</v>
       </c>
       <c r="B151" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C151" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D151" s="10" t="s">
         <v>24</v>
@@ -13289,10 +13421,10 @@
         <v>196</v>
       </c>
       <c r="B155" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C155" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D155" s="10" t="s">
         <v>13</v>
@@ -13541,10 +13673,10 @@
         <v>200</v>
       </c>
       <c r="B159" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C159" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D159" s="10" t="s">
         <v>13</v>
@@ -13793,10 +13925,10 @@
         <v>204</v>
       </c>
       <c r="B163" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C163" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D163" s="10" t="s">
         <v>33</v>
@@ -14045,10 +14177,10 @@
         <v>208</v>
       </c>
       <c r="B167" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C167" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D167" s="10" t="s">
         <v>36</v>
@@ -14297,10 +14429,10 @@
         <v>212</v>
       </c>
       <c r="B171" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C171" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D171" s="10" t="s">
         <v>24</v>
@@ -14549,10 +14681,10 @@
         <v>216</v>
       </c>
       <c r="B175" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C175" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D175" s="10" t="s">
         <v>13</v>
@@ -14801,10 +14933,10 @@
         <v>220</v>
       </c>
       <c r="B179" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C179" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D179" s="10" t="s">
         <v>33</v>
@@ -15053,10 +15185,10 @@
         <v>224</v>
       </c>
       <c r="B183" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C183" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D183" s="10" t="s">
         <v>33</v>
@@ -15305,10 +15437,10 @@
         <v>228</v>
       </c>
       <c r="B187" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C187" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D187" s="10" t="s">
         <v>24</v>
@@ -15557,10 +15689,10 @@
         <v>232</v>
       </c>
       <c r="B191" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C191" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D191" s="10" t="s">
         <v>13</v>
@@ -15809,10 +15941,10 @@
         <v>236</v>
       </c>
       <c r="B195" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C195" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D195" s="10" t="s">
         <v>18</v>
@@ -16061,10 +16193,10 @@
         <v>240</v>
       </c>
       <c r="B199" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C199" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D199" s="10" t="s">
         <v>24</v>
@@ -16313,10 +16445,10 @@
         <v>244</v>
       </c>
       <c r="B203" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C203" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D203" s="10" t="s">
         <v>24</v>
@@ -16565,10 +16697,10 @@
         <v>248</v>
       </c>
       <c r="B207" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C207" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D207" s="10" t="s">
         <v>24</v>
@@ -16817,10 +16949,10 @@
         <v>252</v>
       </c>
       <c r="B211" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C211" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D211" s="10" t="s">
         <v>33</v>
@@ -17069,10 +17201,10 @@
         <v>256</v>
       </c>
       <c r="B215" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C215" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D215" s="10" t="s">
         <v>33</v>
@@ -17321,10 +17453,10 @@
         <v>260</v>
       </c>
       <c r="B219" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C219" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D219" s="10" t="s">
         <v>13</v>
@@ -17573,10 +17705,10 @@
         <v>264</v>
       </c>
       <c r="B223" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C223" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D223" s="10" t="s">
         <v>13</v>
@@ -17825,10 +17957,10 @@
         <v>268</v>
       </c>
       <c r="B227" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C227" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D227" s="10" t="s">
         <v>33</v>
@@ -18077,10 +18209,10 @@
         <v>272</v>
       </c>
       <c r="B231" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C231" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D231" s="10" t="s">
         <v>13</v>
@@ -18329,10 +18461,10 @@
         <v>276</v>
       </c>
       <c r="B235" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C235" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D235" s="10" t="s">
         <v>18</v>
@@ -18581,10 +18713,10 @@
         <v>280</v>
       </c>
       <c r="B239" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C239" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D239" s="10" t="s">
         <v>13</v>
@@ -18833,10 +18965,10 @@
         <v>284</v>
       </c>
       <c r="B243" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C243" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D243" s="10" t="s">
         <v>24</v>
@@ -19085,10 +19217,10 @@
         <v>288</v>
       </c>
       <c r="B247" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C247" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D247" s="10" t="s">
         <v>18</v>
@@ -19337,10 +19469,10 @@
         <v>292</v>
       </c>
       <c r="B251" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C251" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D251" s="10" t="s">
         <v>33</v>
@@ -19589,10 +19721,10 @@
         <v>296</v>
       </c>
       <c r="B255" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C255" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D255" s="10" t="s">
         <v>13</v>
@@ -19841,10 +19973,10 @@
         <v>300</v>
       </c>
       <c r="B259" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C259" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D259" s="10" t="s">
         <v>18</v>
@@ -20093,10 +20225,10 @@
         <v>304</v>
       </c>
       <c r="B263" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C263" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D263" s="10" t="s">
         <v>24</v>
@@ -20345,10 +20477,10 @@
         <v>308</v>
       </c>
       <c r="B267" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C267" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D267" s="10" t="s">
         <v>33</v>
@@ -20597,10 +20729,10 @@
         <v>312</v>
       </c>
       <c r="B271" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C271" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D271" s="10" t="s">
         <v>13</v>
@@ -20849,10 +20981,10 @@
         <v>316</v>
       </c>
       <c r="B275" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C275" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D275" s="10" t="s">
         <v>33</v>
@@ -21101,10 +21233,10 @@
         <v>320</v>
       </c>
       <c r="B279" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C279" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D279" s="10" t="s">
         <v>24</v>
@@ -21353,10 +21485,10 @@
         <v>324</v>
       </c>
       <c r="B283" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C283" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D283" s="10" t="s">
         <v>36</v>
@@ -21605,10 +21737,10 @@
         <v>328</v>
       </c>
       <c r="B287" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C287" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D287" s="10" t="s">
         <v>24</v>
@@ -21857,10 +21989,10 @@
         <v>332</v>
       </c>
       <c r="B291" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C291" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D291" s="10" t="s">
         <v>13</v>
@@ -22109,10 +22241,10 @@
         <v>336</v>
       </c>
       <c r="B295" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C295" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D295" s="10" t="s">
         <v>33</v>
@@ -22361,10 +22493,10 @@
         <v>340</v>
       </c>
       <c r="B299" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C299" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D299" s="10" t="s">
         <v>24</v>
@@ -22613,10 +22745,10 @@
         <v>344</v>
       </c>
       <c r="B303" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C303" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D303" s="10" t="s">
         <v>33</v>
@@ -22865,10 +22997,10 @@
         <v>348</v>
       </c>
       <c r="B307" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C307" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D307" s="10" t="s">
         <v>36</v>
@@ -23117,10 +23249,10 @@
         <v>352</v>
       </c>
       <c r="B311" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C311" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D311" s="10" t="s">
         <v>36</v>
@@ -23369,10 +23501,10 @@
         <v>356</v>
       </c>
       <c r="B315" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C315" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D315" s="10" t="s">
         <v>24</v>
@@ -23621,10 +23753,10 @@
         <v>360</v>
       </c>
       <c r="B319" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C319" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D319" s="10" t="s">
         <v>13</v>
@@ -23873,10 +24005,10 @@
         <v>364</v>
       </c>
       <c r="B323" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C323" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D323" s="10" t="s">
         <v>36</v>
@@ -24125,10 +24257,10 @@
         <v>368</v>
       </c>
       <c r="B327" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C327" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D327" s="10" t="s">
         <v>36</v>
@@ -24377,10 +24509,10 @@
         <v>372</v>
       </c>
       <c r="B331" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C331" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D331" s="10" t="s">
         <v>13</v>
@@ -24629,10 +24761,10 @@
         <v>376</v>
       </c>
       <c r="B335" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C335" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D335" s="10" t="s">
         <v>18</v>
@@ -24881,10 +25013,10 @@
         <v>380</v>
       </c>
       <c r="B339" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C339" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D339" s="10" t="s">
         <v>33</v>
@@ -25133,10 +25265,10 @@
         <v>384</v>
       </c>
       <c r="B343" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C343" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D343" s="10" t="s">
         <v>24</v>
@@ -25385,10 +25517,10 @@
         <v>388</v>
       </c>
       <c r="B347" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C347" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D347" s="10" t="s">
         <v>18</v>
@@ -25637,10 +25769,10 @@
         <v>392</v>
       </c>
       <c r="B351" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C351" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D351" s="10" t="s">
         <v>13</v>
@@ -25889,10 +26021,10 @@
         <v>396</v>
       </c>
       <c r="B355" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C355" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D355" s="10" t="s">
         <v>18</v>
@@ -26141,10 +26273,10 @@
         <v>400</v>
       </c>
       <c r="B359" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C359" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D359" s="10" t="s">
         <v>24</v>
@@ -26393,10 +26525,10 @@
         <v>404</v>
       </c>
       <c r="B363" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C363" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D363" s="10" t="s">
         <v>36</v>
@@ -26645,10 +26777,10 @@
         <v>408</v>
       </c>
       <c r="B367" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C367" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D367" s="10" t="s">
         <v>18</v>
@@ -26897,10 +27029,10 @@
         <v>412</v>
       </c>
       <c r="B371" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C371" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D371" s="10" t="s">
         <v>36</v>
@@ -27149,10 +27281,10 @@
         <v>416</v>
       </c>
       <c r="B375" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C375" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D375" s="10" t="s">
         <v>13</v>
@@ -27401,10 +27533,10 @@
         <v>420</v>
       </c>
       <c r="B379" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C379" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D379" s="10" t="s">
         <v>33</v>
@@ -27653,10 +27785,10 @@
         <v>424</v>
       </c>
       <c r="B383" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C383" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D383" s="10" t="s">
         <v>36</v>
@@ -27905,10 +28037,10 @@
         <v>428</v>
       </c>
       <c r="B387" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C387" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D387" s="10" t="s">
         <v>13</v>
@@ -28157,10 +28289,10 @@
         <v>432</v>
       </c>
       <c r="B391" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C391" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D391" s="10" t="s">
         <v>36</v>
@@ -28409,10 +28541,10 @@
         <v>436</v>
       </c>
       <c r="B395" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C395" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D395" s="10" t="s">
         <v>36</v>
@@ -28661,10 +28793,10 @@
         <v>440</v>
       </c>
       <c r="B399" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C399" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D399" s="10" t="s">
         <v>13</v>
@@ -28913,10 +29045,10 @@
         <v>444</v>
       </c>
       <c r="B403" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C403" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D403" s="10" t="s">
         <v>18</v>
@@ -29165,10 +29297,10 @@
         <v>448</v>
       </c>
       <c r="B407" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C407" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D407" s="10" t="s">
         <v>24</v>
@@ -29417,10 +29549,10 @@
         <v>452</v>
       </c>
       <c r="B411" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C411" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D411" s="10" t="s">
         <v>33</v>
@@ -29669,10 +29801,10 @@
         <v>456</v>
       </c>
       <c r="B415" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C415" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D415" s="10" t="s">
         <v>36</v>
@@ -29921,10 +30053,10 @@
         <v>460</v>
       </c>
       <c r="B419" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C419" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D419" s="10" t="s">
         <v>24</v>
@@ -30173,10 +30305,10 @@
         <v>464</v>
       </c>
       <c r="B423" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C423" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D423" s="10" t="s">
         <v>13</v>
@@ -30425,10 +30557,10 @@
         <v>468</v>
       </c>
       <c r="B427" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C427" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D427" s="10" t="s">
         <v>33</v>
@@ -30677,10 +30809,10 @@
         <v>472</v>
       </c>
       <c r="B431" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C431" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D431" s="10" t="s">
         <v>24</v>
@@ -30929,10 +31061,10 @@
         <v>476</v>
       </c>
       <c r="B435" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C435" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D435" s="10" t="s">
         <v>36</v>
@@ -31181,10 +31313,10 @@
         <v>480</v>
       </c>
       <c r="B439" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C439" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D439" s="10" t="s">
         <v>24</v>
@@ -31433,10 +31565,10 @@
         <v>484</v>
       </c>
       <c r="B443" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C443" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D443" s="10" t="s">
         <v>24</v>
@@ -31685,10 +31817,10 @@
         <v>488</v>
       </c>
       <c r="B447" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C447" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D447" s="10" t="s">
         <v>24</v>
@@ -31937,10 +32069,10 @@
         <v>492</v>
       </c>
       <c r="B451" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C451" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D451" s="10" t="s">
         <v>24</v>
@@ -32189,10 +32321,10 @@
         <v>496</v>
       </c>
       <c r="B455" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C455" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D455" s="10" t="s">
         <v>33</v>
@@ -32441,10 +32573,10 @@
         <v>500</v>
       </c>
       <c r="B459" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C459" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D459" s="10" t="s">
         <v>13</v>
@@ -32693,10 +32825,10 @@
         <v>504</v>
       </c>
       <c r="B463" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C463" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D463" s="10" t="s">
         <v>24</v>
@@ -32945,10 +33077,10 @@
         <v>508</v>
       </c>
       <c r="B467" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C467" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D467" s="10" t="s">
         <v>18</v>
@@ -33197,10 +33329,10 @@
         <v>512</v>
       </c>
       <c r="B471" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C471" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D471" s="10" t="s">
         <v>33</v>
@@ -33449,10 +33581,10 @@
         <v>516</v>
       </c>
       <c r="B475" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C475" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D475" s="10" t="s">
         <v>24</v>
@@ -33701,10 +33833,10 @@
         <v>520</v>
       </c>
       <c r="B479" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C479" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D479" s="10" t="s">
         <v>33</v>
@@ -33953,10 +34085,10 @@
         <v>524</v>
       </c>
       <c r="B483" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C483" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D483" s="10" t="s">
         <v>24</v>
@@ -34205,10 +34337,10 @@
         <v>528</v>
       </c>
       <c r="B487" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C487" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D487" s="10" t="s">
         <v>36</v>
@@ -34457,10 +34589,10 @@
         <v>532</v>
       </c>
       <c r="B491" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C491" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D491" s="10" t="s">
         <v>24</v>
@@ -34709,10 +34841,10 @@
         <v>536</v>
       </c>
       <c r="B495" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C495" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D495" s="10" t="s">
         <v>36</v>
@@ -34961,10 +35093,10 @@
         <v>540</v>
       </c>
       <c r="B499" s="9" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C499" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D499" s="10" t="s">
         <v>33</v>
@@ -35103,7 +35235,7 @@
     <row r="503" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A503" s="1"/>
       <c r="B503" s="25" t="s">
-        <v>688</v>
+        <v>684</v>
       </c>
       <c r="C503" s="1">
         <f>SUM(Sales)</f>
@@ -35135,7 +35267,7 @@
     <row r="504" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A504" s="1"/>
       <c r="B504" s="25" t="s">
-        <v>689</v>
+        <v>685</v>
       </c>
       <c r="C504" s="1" cm="1">
         <f t="array" ref="C504">SUBTOTAL(9,Sales)</f>
@@ -48557,7 +48689,7 @@
       <c r="Y1000" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="9" type="noConversion"/>
   <conditionalFormatting sqref="E1:F1048576">
     <cfRule type="top10" dxfId="4" priority="5" bottom="1" rank="10"/>
     <cfRule type="top10" dxfId="3" priority="6" rank="10"/>
@@ -48579,11 +48711,551 @@
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R50" xr:uid="{7D061CD3-32D3-4A49-A982-879635F5FEBC}">
+      <formula1>$A$2:$A$499</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
   <tableParts count="1">
     <tablePart r:id="rId2"/>
   </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D425F623-917B-4F49-855A-1B9221A6FFAC}">
+  <dimension ref="A3:G14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="34"/>
+      <c r="B3" s="34" t="s">
+        <v>693</v>
+      </c>
+      <c r="C3" s="34" t="s">
+        <v>694</v>
+      </c>
+      <c r="D3" s="34" t="s">
+        <v>695</v>
+      </c>
+      <c r="E3" s="34" t="s">
+        <v>696</v>
+      </c>
+      <c r="F3" s="34" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="34" t="s">
+        <v>697</v>
+      </c>
+      <c r="B4" s="34">
+        <v>100</v>
+      </c>
+      <c r="C4" s="34">
+        <v>585</v>
+      </c>
+      <c r="D4" s="34">
+        <v>333</v>
+      </c>
+      <c r="E4" s="34">
+        <v>745</v>
+      </c>
+      <c r="F4" s="34">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="34" t="s">
+        <v>698</v>
+      </c>
+      <c r="B5" s="34">
+        <v>100</v>
+      </c>
+      <c r="C5" s="34">
+        <v>500</v>
+      </c>
+      <c r="D5" s="34">
+        <v>600</v>
+      </c>
+      <c r="E5" s="34">
+        <v>700</v>
+      </c>
+      <c r="F5" s="34">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="34" t="s">
+        <v>572</v>
+      </c>
+      <c r="B6" s="34">
+        <v>2000</v>
+      </c>
+      <c r="C6" s="34">
+        <v>7000</v>
+      </c>
+      <c r="D6" s="34">
+        <v>8000</v>
+      </c>
+      <c r="E6" s="34">
+        <v>6000</v>
+      </c>
+      <c r="F6" s="34">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="34" t="s">
+        <v>699</v>
+      </c>
+      <c r="B7" s="34">
+        <v>400</v>
+      </c>
+      <c r="C7" s="34">
+        <v>500</v>
+      </c>
+      <c r="D7" s="34">
+        <v>300</v>
+      </c>
+      <c r="E7" s="34">
+        <v>300</v>
+      </c>
+      <c r="F7" s="34">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B11" s="34" t="s">
+        <v>700</v>
+      </c>
+      <c r="C11" s="34" t="s">
+        <v>694</v>
+      </c>
+      <c r="F11" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B12" s="34" t="s">
+        <v>572</v>
+      </c>
+      <c r="C12" s="34">
+        <f>HLOOKUP($C$11,$B$3:$F$7,MATCH(B12,$A$3:$A$7,0),FALSE)</f>
+        <v>7000</v>
+      </c>
+      <c r="F12" s="34" t="s">
+        <v>700</v>
+      </c>
+      <c r="G12" s="34" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B13" s="34" t="s">
+        <v>698</v>
+      </c>
+      <c r="C13" s="34">
+        <f>HLOOKUP($C$11,$B$3:$F$7,MATCH(B13,$A$3:$A$7,0),FALSE)</f>
+        <v>500</v>
+      </c>
+      <c r="F13" s="34" t="s">
+        <v>572</v>
+      </c>
+      <c r="G13" s="34">
+        <f>VLOOKUP(F13,$A$4:$F$7,MATCH($F$3,$A$3:$F$3,0),FALSE)</f>
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B14" s="34" t="s">
+        <v>699</v>
+      </c>
+      <c r="C14" s="34">
+        <f>HLOOKUP($C$11,$B$3:$F$7,MATCH(B14,$A$3:$A$7,0),FALSE)</f>
+        <v>500</v>
+      </c>
+      <c r="F14" s="34" t="s">
+        <v>699</v>
+      </c>
+      <c r="G14" s="34">
+        <f>VLOOKUP(F14,$A$4:$F$7,MATCH($F$3,$A$3:$F$3,0),FALSE)</f>
+        <v>200</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="9" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFDEB056-8791-4327-A9B4-16DDB7F517A1}">
+  <dimension ref="A1:T13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="11.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A1" s="34"/>
+      <c r="B1" s="66" t="s">
+        <v>641</v>
+      </c>
+      <c r="C1" s="66" t="s">
+        <v>705</v>
+      </c>
+      <c r="D1" s="66" t="s">
+        <v>706</v>
+      </c>
+      <c r="E1" s="66"/>
+      <c r="G1" s="67" t="s">
+        <v>712</v>
+      </c>
+      <c r="H1" s="67" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A2" s="66" t="s">
+        <v>707</v>
+      </c>
+      <c r="B2" s="34">
+        <v>55</v>
+      </c>
+      <c r="C2" s="34">
+        <v>44</v>
+      </c>
+      <c r="D2" s="34">
+        <v>44</v>
+      </c>
+      <c r="E2" s="34"/>
+      <c r="G2" t="s">
+        <v>713</v>
+      </c>
+      <c r="H2" t="e" cm="1">
+        <f t="array" aca="1" ref="H2" ca="1">SUM(H1,INDIRECT(Lemons))</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Q2">
+        <v>34</v>
+      </c>
+      <c r="R2" t="s">
+        <v>703</v>
+      </c>
+      <c r="T2" cm="1">
+        <f t="array" aca="1" ref="T2" ca="1">INDIRECT("B2")</f>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A3" s="66" t="s">
+        <v>708</v>
+      </c>
+      <c r="B3" s="34">
+        <v>33</v>
+      </c>
+      <c r="C3" s="34">
+        <v>32</v>
+      </c>
+      <c r="D3" s="34">
+        <v>66</v>
+      </c>
+      <c r="E3" s="34"/>
+      <c r="G3" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A4" s="66" t="s">
+        <v>709</v>
+      </c>
+      <c r="B4" s="34">
+        <v>45</v>
+      </c>
+      <c r="C4" s="34">
+        <v>50</v>
+      </c>
+      <c r="D4" s="34">
+        <v>44</v>
+      </c>
+      <c r="E4" s="34"/>
+      <c r="G4" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A5" s="66" t="s">
+        <v>710</v>
+      </c>
+      <c r="B5" s="34">
+        <v>34</v>
+      </c>
+      <c r="C5" s="34">
+        <v>32</v>
+      </c>
+      <c r="D5" s="34">
+        <v>22</v>
+      </c>
+      <c r="E5" s="34"/>
+      <c r="G5" t="s">
+        <v>716</v>
+      </c>
+      <c r="Q5">
+        <v>54</v>
+      </c>
+      <c r="R5" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A6" s="66" t="s">
+        <v>711</v>
+      </c>
+      <c r="B6" s="34">
+        <v>21</v>
+      </c>
+      <c r="C6" s="34">
+        <v>26</v>
+      </c>
+      <c r="D6" s="34">
+        <v>66</v>
+      </c>
+      <c r="E6" s="34"/>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="P7" t="s">
+        <v>548</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>549</v>
+      </c>
+      <c r="R7" t="str">
+        <f>P7&amp;" "&amp;Q7</f>
+        <v>Suhas Borkar</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="H8" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="D9" cm="1">
+        <f t="array" aca="1" ref="D9:D13" ca="1">INDIRECT(B1,TRUE)</f>
+        <v>55</v>
+      </c>
+      <c r="F9" cm="1">
+        <f t="array" aca="1" ref="F9" ca="1">INDIRECT("D9",TRUE)</f>
+        <v>55</v>
+      </c>
+      <c r="H9" cm="1">
+        <f t="array" aca="1" ref="H9" ca="1">INDIRECT("R9C4",FALSE)</f>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="D10">
+        <f ca="1"/>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="D11">
+        <f ca="1"/>
+        <v>45</v>
+      </c>
+      <c r="G11" t="str" cm="1">
+        <f t="array" aca="1" ref="G11" ca="1">INDIRECT("R1C2",FALSE)</f>
+        <v>Apples</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="D12">
+        <f ca="1"/>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="D13">
+        <f ca="1"/>
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B8F3A29-5C2F-43FF-B757-CC928EEFA7EF}">
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="13.109375" style="71" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="66" t="s">
+        <v>717</v>
+      </c>
+      <c r="B1" s="75" t="s">
+        <v>724</v>
+      </c>
+      <c r="C1" s="66" t="s">
+        <v>718</v>
+      </c>
+      <c r="D1" s="66" t="s">
+        <v>721</v>
+      </c>
+      <c r="E1" s="73" t="s">
+        <v>604</v>
+      </c>
+      <c r="F1" s="74" t="s">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" s="34">
+        <v>21</v>
+      </c>
+      <c r="B2" s="34">
+        <v>1425</v>
+      </c>
+      <c r="C2" s="34">
+        <v>2</v>
+      </c>
+      <c r="D2" s="70">
+        <v>45262</v>
+      </c>
+      <c r="E2" s="34">
+        <v>41</v>
+      </c>
+      <c r="F2" s="68"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" s="34">
+        <v>18</v>
+      </c>
+      <c r="B3" s="76" t="s">
+        <v>725</v>
+      </c>
+      <c r="C3" s="34">
+        <v>10</v>
+      </c>
+      <c r="D3" s="70">
+        <v>46218</v>
+      </c>
+      <c r="E3" s="34"/>
+      <c r="F3" s="68"/>
+      <c r="I3" t="s">
+        <v>719</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3" s="72" t="s">
+        <v>722</v>
+      </c>
+      <c r="L3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" s="34">
+        <v>12</v>
+      </c>
+      <c r="B4" s="34"/>
+      <c r="C4" s="34">
+        <v>5</v>
+      </c>
+      <c r="D4" s="70"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="68"/>
+      <c r="I4" t="s">
+        <v>720</v>
+      </c>
+      <c r="J4">
+        <v>10</v>
+      </c>
+      <c r="K4" s="72" t="s">
+        <v>723</v>
+      </c>
+      <c r="L4">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" s="34">
+        <v>20</v>
+      </c>
+      <c r="B5" s="34"/>
+      <c r="C5" s="34">
+        <v>6</v>
+      </c>
+      <c r="D5" s="70"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="68"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" s="34">
+        <v>25</v>
+      </c>
+      <c r="B6" s="34"/>
+      <c r="C6" s="34">
+        <v>5</v>
+      </c>
+      <c r="D6" s="70"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="68"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7" s="69">
+        <v>25</v>
+      </c>
+      <c r="B7" s="69"/>
+      <c r="C7" s="69">
+        <v>9</v>
+      </c>
+      <c r="D7" s="70"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="68"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" s="69">
+        <v>12</v>
+      </c>
+      <c r="B8" s="69"/>
+      <c r="C8" s="69">
+        <v>8</v>
+      </c>
+      <c r="D8" s="70"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="68"/>
+    </row>
+  </sheetData>
+  <dataValidations count="5">
+    <dataValidation type="whole" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Age Error" error="The age entered is not within range" promptTitle="Age Restrictions" prompt="Enter Age betweeen 18 to 60" sqref="A1:A1048576" xr:uid="{F3825B10-C281-46CF-9164-2019892889DD}">
+      <formula1>18</formula1>
+      <formula2>60</formula2>
+    </dataValidation>
+    <dataValidation type="date" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Wrong Date" error="You have entred wrong date" promptTitle="DATE" prompt="Enter Date " sqref="D2:D1048576" xr:uid="{EBC0259C-BFAE-49C7-B81A-B5154ED856B3}">
+      <formula1>46218</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:F1048576" xr:uid="{FC2D94F4-7FE8-43E6-8531-397E2DB3E9E1}">
+      <formula1>AND(E2&gt;40,E2&lt;=75)</formula1>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Wrong Quantity" error="Entered Value is wrong" promptTitle="Quantity" prompt="Enter quantity in 2 to 10" sqref="C2:C1048576" xr:uid="{9053FF0A-56C9-4C65-BBA0-B7C8036D947A}">
+      <formula1>$J$3</formula1>
+      <formula2>$J$4</formula2>
+    </dataValidation>
+    <dataValidation type="textLength" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="INCORRECT OTP" error="You have entered wrong OTP_x000a_" promptTitle="OTP" prompt="Enter the OTP ( 4 CHAR )" sqref="B2:B1048576" xr:uid="{F96F00EF-7913-44F2-B72A-14291EFFAF41}">
+      <formula1>4</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -48604,24 +49276,24 @@
         <v>1</v>
       </c>
       <c r="C2" s="46" t="s">
-        <v>637</v>
+        <v>633</v>
       </c>
       <c r="D2" s="46" t="s">
-        <v>576</v>
+        <v>572</v>
       </c>
     </row>
     <row r="3" spans="2:8" ht="15" x14ac:dyDescent="0.3">
       <c r="B3" s="47" t="s">
-        <v>638</v>
+        <v>634</v>
       </c>
       <c r="C3" s="47" t="s">
-        <v>639</v>
+        <v>635</v>
       </c>
       <c r="D3" s="48">
         <v>2300</v>
       </c>
       <c r="G3" s="49" t="s">
-        <v>646</v>
+        <v>642</v>
       </c>
       <c r="H3">
         <f>SUMIF(B3:B10,"Fruits",D3:D10)</f>
@@ -48630,16 +49302,16 @@
     </row>
     <row r="4" spans="2:8" ht="15" x14ac:dyDescent="0.3">
       <c r="B4" s="47" t="s">
-        <v>638</v>
+        <v>634</v>
       </c>
       <c r="C4" s="47" t="s">
-        <v>640</v>
+        <v>636</v>
       </c>
       <c r="D4" s="48">
         <v>5500</v>
       </c>
       <c r="G4" s="49" t="s">
-        <v>647</v>
+        <v>643</v>
       </c>
       <c r="H4">
         <f>SUMIF(B3:B10,"Vegetables",D3:D10)</f>
@@ -48648,16 +49320,16 @@
     </row>
     <row r="5" spans="2:8" ht="15" x14ac:dyDescent="0.3">
       <c r="B5" s="47" t="s">
-        <v>641</v>
+        <v>637</v>
       </c>
       <c r="C5" s="47" t="s">
-        <v>642</v>
+        <v>638</v>
       </c>
       <c r="D5" s="48">
         <v>800</v>
       </c>
       <c r="G5" s="49" t="s">
-        <v>648</v>
+        <v>644</v>
       </c>
       <c r="H5">
         <f>SUMIF(B3:B10,"",D3:D10)</f>
@@ -48667,7 +49339,7 @@
     <row r="6" spans="2:8" ht="15" x14ac:dyDescent="0.3">
       <c r="B6" s="47"/>
       <c r="C6" s="47" t="s">
-        <v>643</v>
+        <v>639</v>
       </c>
       <c r="D6" s="48">
         <v>400</v>
@@ -48675,10 +49347,10 @@
     </row>
     <row r="7" spans="2:8" ht="15" x14ac:dyDescent="0.3">
       <c r="B7" s="47" t="s">
-        <v>638</v>
+        <v>634</v>
       </c>
       <c r="C7" s="47" t="s">
-        <v>644</v>
+        <v>640</v>
       </c>
       <c r="D7" s="48">
         <v>4200</v>
@@ -48687,7 +49359,7 @@
     <row r="8" spans="2:8" ht="15" x14ac:dyDescent="0.3">
       <c r="B8" s="47"/>
       <c r="C8" s="47" t="s">
-        <v>649</v>
+        <v>645</v>
       </c>
       <c r="D8" s="48">
         <v>1000</v>
@@ -48696,7 +49368,7 @@
     <row r="9" spans="2:8" ht="15" x14ac:dyDescent="0.3">
       <c r="B9" s="47"/>
       <c r="C9" s="47" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="D9" s="48">
         <v>500</v>
@@ -48704,10 +49376,10 @@
     </row>
     <row r="10" spans="2:8" ht="15" x14ac:dyDescent="0.3">
       <c r="B10" s="47" t="s">
+        <v>637</v>
+      </c>
+      <c r="C10" s="47" t="s">
         <v>641</v>
-      </c>
-      <c r="C10" s="47" t="s">
-        <v>645</v>
       </c>
       <c r="D10" s="48">
         <v>1200</v>
@@ -48728,6 +49400,7 @@
     <col min="3" max="3" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -48750,7 +49423,7 @@
         <v>568</v>
       </c>
       <c r="G1" t="s">
-        <v>573</v>
+        <v>569</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
@@ -48769,8 +49442,11 @@
       <c r="E2" t="s">
         <v>565</v>
       </c>
-      <c r="F2" t="s">
-        <v>569</v>
+      <c r="F2">
+        <v>91</v>
+      </c>
+      <c r="G2">
+        <v>8967598967</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -48789,8 +49465,11 @@
       <c r="E3" t="s">
         <v>566</v>
       </c>
-      <c r="F3" t="s">
-        <v>570</v>
+      <c r="F3">
+        <v>91</v>
+      </c>
+      <c r="G3">
+        <v>9878586967</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -48809,8 +49488,11 @@
       <c r="E4" t="s">
         <v>563</v>
       </c>
-      <c r="F4" t="s">
-        <v>571</v>
+      <c r="F4">
+        <v>91</v>
+      </c>
+      <c r="G4">
+        <v>9089788767</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -48829,8 +49511,11 @@
       <c r="E5" t="s">
         <v>567</v>
       </c>
-      <c r="F5" t="s">
-        <v>572</v>
+      <c r="F5">
+        <v>91</v>
+      </c>
+      <c r="G5">
+        <v>8978877890</v>
       </c>
     </row>
   </sheetData>
@@ -48860,38 +49545,38 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
-        <v>581</v>
+        <v>577</v>
       </c>
       <c r="C1" s="28" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="D1" s="28" t="s">
-        <v>576</v>
+        <v>572</v>
       </c>
       <c r="E1" s="28" t="s">
+        <v>591</v>
+      </c>
+      <c r="G1" s="28" t="s">
+        <v>593</v>
+      </c>
+      <c r="H1" s="28" t="s">
+        <v>594</v>
+      </c>
+      <c r="I1" s="28" t="s">
         <v>595</v>
       </c>
-      <c r="G1" s="28" t="s">
+      <c r="J1" s="28" t="s">
+        <v>596</v>
+      </c>
+      <c r="K1" s="28" t="s">
         <v>597</v>
-      </c>
-      <c r="H1" s="28" t="s">
-        <v>598</v>
-      </c>
-      <c r="I1" s="28" t="s">
-        <v>599</v>
-      </c>
-      <c r="J1" s="28" t="s">
-        <v>600</v>
-      </c>
-      <c r="K1" s="28" t="s">
-        <v>601</v>
       </c>
       <c r="L1" s="28"/>
       <c r="O1" s="29" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="P1" s="29" t="s">
-        <v>576</v>
+        <v>572</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
@@ -48899,7 +49584,7 @@
         <v>548</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="D2">
         <v>23454</v>
@@ -48925,7 +49610,7 @@
         <v>A</v>
       </c>
       <c r="O2" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="P2">
         <v>23454</v>
@@ -48933,10 +49618,10 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="26" t="s">
-        <v>578</v>
+        <v>574</v>
       </c>
       <c r="C3" s="26" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="D3">
         <v>56567</v>
@@ -48945,7 +49630,7 @@
         <v>Yes</v>
       </c>
       <c r="G3" s="26" t="s">
-        <v>579</v>
+        <v>575</v>
       </c>
       <c r="H3">
         <v>98</v>
@@ -48961,7 +49646,7 @@
         <v>A</v>
       </c>
       <c r="O3" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="P3">
         <v>56567</v>
@@ -48969,10 +49654,10 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="26" t="s">
+        <v>575</v>
+      </c>
+      <c r="C4" s="26" t="s">
         <v>579</v>
-      </c>
-      <c r="C4" s="26" t="s">
-        <v>583</v>
       </c>
       <c r="D4">
         <v>76856</v>
@@ -48981,7 +49666,7 @@
         <v>Yes</v>
       </c>
       <c r="G4" s="26" t="s">
-        <v>602</v>
+        <v>598</v>
       </c>
       <c r="H4">
         <v>98</v>
@@ -48997,7 +49682,7 @@
         <v>A+</v>
       </c>
       <c r="O4" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
       <c r="P4">
         <v>76856</v>
@@ -49005,10 +49690,10 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" s="26" t="s">
+        <v>576</v>
+      </c>
+      <c r="C5" s="26" t="s">
         <v>580</v>
-      </c>
-      <c r="C5" s="26" t="s">
-        <v>584</v>
       </c>
       <c r="D5">
         <v>76756</v>
@@ -49017,7 +49702,7 @@
         <v>Yes</v>
       </c>
       <c r="O5" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
       <c r="P5">
         <v>76756</v>
@@ -49025,7 +49710,7 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C6" s="26" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="D6">
         <v>56456</v>
@@ -49034,7 +49719,7 @@
         <v>Yes</v>
       </c>
       <c r="O6" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="P6">
         <v>56456</v>
@@ -49042,7 +49727,7 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C7" s="26" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="D7">
         <v>67645</v>
@@ -49051,16 +49736,16 @@
         <v>Yes</v>
       </c>
       <c r="H7" s="26" t="s">
-        <v>603</v>
+        <v>599</v>
       </c>
       <c r="I7" s="26" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="J7" s="26" t="s">
-        <v>606</v>
+        <v>602</v>
       </c>
       <c r="O7" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="P7">
         <v>67645</v>
@@ -49068,7 +49753,7 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C8" s="26" t="s">
-        <v>589</v>
+        <v>585</v>
       </c>
       <c r="D8">
         <v>49000</v>
@@ -49077,10 +49762,10 @@
         <v>No</v>
       </c>
       <c r="H8" s="26" t="s">
-        <v>605</v>
+        <v>601</v>
       </c>
       <c r="O8" t="s">
-        <v>589</v>
+        <v>585</v>
       </c>
       <c r="P8">
         <v>65589</v>
@@ -49088,7 +49773,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C10" s="26" t="s">
-        <v>596</v>
+        <v>592</v>
       </c>
       <c r="D10">
         <v>50000</v>
@@ -49096,16 +49781,16 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="G11" s="30" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
       <c r="H11" s="30" t="s">
+        <v>603</v>
+      </c>
+      <c r="I11" s="30" t="s">
+        <v>604</v>
+      </c>
+      <c r="J11" s="30" t="s">
         <v>607</v>
-      </c>
-      <c r="I11" s="30" t="s">
-        <v>608</v>
-      </c>
-      <c r="J11" s="30" t="s">
-        <v>611</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
@@ -49113,7 +49798,7 @@
         <v>548</v>
       </c>
       <c r="H12" s="26" t="s">
-        <v>609</v>
+        <v>605</v>
       </c>
       <c r="I12">
         <v>90</v>
@@ -49125,7 +49810,7 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="G13" s="26" t="s">
-        <v>579</v>
+        <v>575</v>
       </c>
       <c r="H13" s="26" t="s">
         <v>26</v>
@@ -49140,10 +49825,10 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="G14" s="26" t="s">
-        <v>602</v>
+        <v>598</v>
       </c>
       <c r="H14" s="26" t="s">
-        <v>610</v>
+        <v>606</v>
       </c>
       <c r="I14">
         <v>78</v>
@@ -49153,7 +49838,7 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C2:D8">
     <sortCondition ref="C2:C8" customList="January,February,March,April,May,June,July,August,September,October,November,December"/>
   </sortState>
-  <phoneticPr fontId="14" type="noConversion"/>
+  <phoneticPr fontId="15" type="noConversion"/>
   <conditionalFormatting sqref="D2:D8">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
       <formula>50000</formula>
@@ -49180,45 +49865,45 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="26" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="26" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="26" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="26" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="26" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="D5" s="34" t="s">
+        <v>673</v>
+      </c>
+      <c r="E5" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="F5" s="60" t="s">
         <v>677</v>
-      </c>
-      <c r="E5" s="33" t="s">
-        <v>577</v>
-      </c>
-      <c r="F5" s="60" t="s">
-        <v>681</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="26" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="C6" s="26"/>
       <c r="D6" s="34" t="s">
-        <v>678</v>
+        <v>674</v>
       </c>
       <c r="E6" s="59" t="s">
         <v>548</v>
@@ -49227,7 +49912,7 @@
         <v>1001</v>
       </c>
       <c r="H6" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="I6">
         <f>COUNTIF(F6:F10,F7)</f>
@@ -49236,19 +49921,19 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="26" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="D7" s="34" t="s">
-        <v>679</v>
+        <v>675</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>578</v>
+        <v>574</v>
       </c>
       <c r="F7">
         <v>1002</v>
       </c>
       <c r="H7" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="I7">
         <f>COUNTIF(E6:E10,"Suhas")</f>
@@ -49257,13 +49942,13 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="26" t="s">
-        <v>591</v>
+        <v>587</v>
       </c>
       <c r="D8" s="34" t="s">
-        <v>680</v>
+        <v>676</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>579</v>
+        <v>575</v>
       </c>
       <c r="F8">
         <v>1003</v>
@@ -49271,13 +49956,13 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="26" t="s">
-        <v>589</v>
+        <v>585</v>
       </c>
       <c r="D9" s="34" t="s">
+        <v>572</v>
+      </c>
+      <c r="E9" s="33" t="s">
         <v>576</v>
-      </c>
-      <c r="E9" s="33" t="s">
-        <v>580</v>
       </c>
       <c r="F9">
         <v>1001</v>
@@ -49285,10 +49970,10 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="26" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="D10" s="34" t="s">
-        <v>678</v>
+        <v>674</v>
       </c>
       <c r="E10" s="58" t="s">
         <v>548</v>
@@ -49299,16 +49984,16 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="26" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="26" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="14" type="noConversion"/>
+  <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -49327,19 +50012,19 @@
   <sheetData>
     <row r="3" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B3" s="32" t="s">
+        <v>593</v>
+      </c>
+      <c r="C3" s="32" t="s">
+        <v>604</v>
+      </c>
+      <c r="D3" s="32" t="s">
         <v>597</v>
       </c>
-      <c r="C3" s="32" t="s">
+      <c r="F3" s="37" t="s">
         <v>608</v>
       </c>
-      <c r="D3" s="32" t="s">
-        <v>601</v>
-      </c>
-      <c r="F3" s="37" t="s">
-        <v>612</v>
-      </c>
       <c r="G3" s="38" t="s">
-        <v>615</v>
+        <v>611</v>
       </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.3">
@@ -49354,15 +50039,15 @@
         <v>A++</v>
       </c>
       <c r="F4" s="39" t="s">
-        <v>613</v>
+        <v>609</v>
       </c>
       <c r="G4" s="40" t="s">
-        <v>603</v>
+        <v>599</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B5" s="33" t="s">
-        <v>579</v>
+        <v>575</v>
       </c>
       <c r="C5" s="34">
         <v>36</v>
@@ -49372,15 +50057,15 @@
         <v>Fail</v>
       </c>
       <c r="F5" s="39" t="s">
-        <v>614</v>
+        <v>610</v>
       </c>
       <c r="G5" s="40" t="s">
-        <v>616</v>
+        <v>612</v>
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B6" s="33" t="s">
-        <v>602</v>
+        <v>598</v>
       </c>
       <c r="C6" s="34">
         <v>88</v>
@@ -49390,10 +50075,10 @@
         <v>A+</v>
       </c>
       <c r="F6" s="39" t="s">
-        <v>617</v>
+        <v>613</v>
       </c>
       <c r="G6" s="40" t="s">
-        <v>605</v>
+        <v>601</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.3">
@@ -49408,15 +50093,15 @@
         <v>B</v>
       </c>
       <c r="F7" s="41" t="s">
-        <v>618</v>
+        <v>614</v>
       </c>
       <c r="G7" s="42" t="s">
-        <v>619</v>
+        <v>615</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B8" s="35" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="C8" s="34">
         <v>62</v>
@@ -49428,22 +50113,22 @@
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B12" s="32" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
       <c r="C12" s="32" t="s">
-        <v>576</v>
+        <v>572</v>
       </c>
       <c r="D12" s="32" t="s">
+        <v>617</v>
+      </c>
+      <c r="E12" s="32" t="s">
+        <v>620</v>
+      </c>
+      <c r="G12" s="37" t="s">
         <v>621</v>
       </c>
-      <c r="E12" s="32" t="s">
-        <v>624</v>
-      </c>
-      <c r="G12" s="37" t="s">
-        <v>625</v>
-      </c>
       <c r="H12" s="38" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.3">
@@ -49470,7 +50155,7 @@
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B14" s="33" t="s">
-        <v>579</v>
+        <v>575</v>
       </c>
       <c r="C14" s="34">
         <v>50000</v>
@@ -49492,7 +50177,7 @@
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B15" s="33" t="s">
-        <v>602</v>
+        <v>598</v>
       </c>
       <c r="C15" s="34">
         <v>45000</v>
@@ -49528,15 +50213,15 @@
         <v>11250</v>
       </c>
       <c r="G16" s="41" t="s">
-        <v>622</v>
+        <v>618</v>
       </c>
       <c r="H16" s="42" t="s">
-        <v>623</v>
+        <v>619</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" s="35" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="C17" s="34">
         <v>55000</v>
@@ -49552,7 +50237,7 @@
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="D19" s="27" t="s">
-        <v>633</v>
+        <v>629</v>
       </c>
       <c r="E19">
         <f>SUMIF(C13:C17,"&gt;50000",C13:C17)</f>
@@ -49561,13 +50246,13 @@
     </row>
     <row r="34" spans="4:6" x14ac:dyDescent="0.3">
       <c r="D34" s="31" t="s">
-        <v>626</v>
+        <v>622</v>
       </c>
       <c r="E34" s="31" t="s">
-        <v>627</v>
+        <v>623</v>
       </c>
       <c r="F34" s="31" t="s">
-        <v>628</v>
+        <v>624</v>
       </c>
     </row>
     <row r="35" spans="4:6" x14ac:dyDescent="0.3">
@@ -49635,7 +50320,7 @@
     <row r="1" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:10" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="62" t="s">
-        <v>683</v>
+        <v>679</v>
       </c>
     </row>
     <row r="3" spans="2:10" ht="16.8" x14ac:dyDescent="0.3">
@@ -49643,10 +50328,10 @@
         <v>120</v>
       </c>
       <c r="E3" s="60" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="I3" s="60" t="s">
-        <v>687</v>
+        <v>683</v>
       </c>
     </row>
     <row r="4" spans="2:10" ht="16.8" x14ac:dyDescent="0.3">
@@ -49659,14 +50344,14 @@
         <v>150</v>
       </c>
       <c r="D5" s="60" t="s">
-        <v>684</v>
+        <v>680</v>
       </c>
       <c r="E5">
         <f>SUBTOTAL(9,B3:B9)</f>
         <v>469</v>
       </c>
       <c r="I5" s="60" t="s">
-        <v>686</v>
+        <v>682</v>
       </c>
       <c r="J5">
         <f>SUBTOTAL(109,B3:B9)</f>
@@ -49723,19 +50408,19 @@
   <sheetData>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="32" t="s">
-        <v>690</v>
+        <v>686</v>
       </c>
       <c r="B2" s="32" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
       <c r="C2" s="32" t="s">
-        <v>576</v>
+        <v>572</v>
       </c>
       <c r="D2" s="32" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="E2" s="32" t="s">
-        <v>624</v>
+        <v>620</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -49762,7 +50447,7 @@
         <v>1002</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>579</v>
+        <v>575</v>
       </c>
       <c r="C4" s="34">
         <v>50000</v>
@@ -49781,7 +50466,7 @@
         <v>1003</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>602</v>
+        <v>598</v>
       </c>
       <c r="C5" s="34">
         <v>45000</v>
@@ -49819,7 +50504,7 @@
         <v>1005</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="C7" s="34">
         <v>55000</v>
@@ -49835,24 +50520,24 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B9" s="27" t="s">
-        <v>694</v>
+        <v>690</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B10" s="65" t="s">
-        <v>691</v>
+        <v>687</v>
       </c>
       <c r="C10" s="65" t="s">
-        <v>576</v>
+        <v>572</v>
       </c>
       <c r="D10" s="65" t="s">
-        <v>624</v>
+        <v>620</v>
       </c>
       <c r="F10" s="65" t="s">
-        <v>692</v>
+        <v>688</v>
       </c>
       <c r="G10" s="65" t="s">
-        <v>693</v>
+        <v>689</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -49868,7 +50553,7 @@
         <v>6750</v>
       </c>
       <c r="F11" t="s">
-        <v>602</v>
+        <v>598</v>
       </c>
       <c r="G11">
         <f>MATCH(F11,B2:B7,0)</f>
@@ -49877,18 +50562,18 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B13" s="27" t="s">
-        <v>695</v>
+        <v>691</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B14" s="65" t="s">
-        <v>691</v>
+        <v>687</v>
       </c>
       <c r="C14" s="65" t="s">
-        <v>576</v>
+        <v>572</v>
       </c>
       <c r="D14" s="65" t="s">
-        <v>624</v>
+        <v>620</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
@@ -49905,7 +50590,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="14" type="noConversion"/>
+  <phoneticPr fontId="15" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B11 B15" xr:uid="{4A439758-2AD6-4796-909D-A3AB5C5BB3DD}">
       <formula1>$A$3:$A$7</formula1>
@@ -49913,4 +50598,157 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E680945C-6A01-49F1-A32C-2F45537581FF}">
+  <dimension ref="B3:G11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B3" s="32" t="s">
+        <v>686</v>
+      </c>
+      <c r="C3" s="33">
+        <v>1001</v>
+      </c>
+      <c r="D3" s="33">
+        <v>1002</v>
+      </c>
+      <c r="E3" s="33">
+        <v>1003</v>
+      </c>
+      <c r="F3" s="35">
+        <v>1004</v>
+      </c>
+      <c r="G3" s="35">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B4" s="32" t="s">
+        <v>593</v>
+      </c>
+      <c r="C4" s="33" t="s">
+        <v>548</v>
+      </c>
+      <c r="D4" s="33" t="s">
+        <v>575</v>
+      </c>
+      <c r="E4" s="33" t="s">
+        <v>598</v>
+      </c>
+      <c r="F4" s="35" t="s">
+        <v>546</v>
+      </c>
+      <c r="G4" s="35" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B5" s="32" t="s">
+        <v>572</v>
+      </c>
+      <c r="C5" s="34">
+        <v>70000</v>
+      </c>
+      <c r="D5" s="34">
+        <v>50000</v>
+      </c>
+      <c r="E5" s="34">
+        <v>45000</v>
+      </c>
+      <c r="F5" s="34">
+        <v>75000</v>
+      </c>
+      <c r="G5" s="34">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B6" s="32" t="s">
+        <v>617</v>
+      </c>
+      <c r="C6" s="36">
+        <f>IF(C5&gt;=$G$13,15%,IF(C5&gt;=$G$14,10%,IF(C5&gt;=$G$15,5%,0%)))</f>
+        <v>0.15</v>
+      </c>
+      <c r="D6" s="36">
+        <f>IF(D5&gt;=$G$13,15%,IF(D5&gt;=$G$14,10%,IF(D5&gt;=$G$15,5%,0%)))</f>
+        <v>0.15</v>
+      </c>
+      <c r="E6" s="36">
+        <f>IF(E5&gt;=$G$13,15%,IF(E5&gt;=$G$14,10%,IF(E5&gt;=$G$15,5%,0%)))</f>
+        <v>0.15</v>
+      </c>
+      <c r="F6" s="36">
+        <f>IF(F5&gt;=$G$13,15%,IF(F5&gt;=$G$14,10%,IF(F5&gt;=$G$15,5%,0%)))</f>
+        <v>0.15</v>
+      </c>
+      <c r="G6" s="36">
+        <f>IF(G5&gt;=$G$13,15%,IF(G5&gt;=$G$14,10%,IF(G5&gt;=$G$15,5%,0%)))</f>
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B7" s="32" t="s">
+        <v>620</v>
+      </c>
+      <c r="C7" s="34">
+        <f>C5*C6</f>
+        <v>10500</v>
+      </c>
+      <c r="D7" s="34">
+        <f>D5*D6</f>
+        <v>7500</v>
+      </c>
+      <c r="E7" s="34">
+        <f>E5*E6</f>
+        <v>6750</v>
+      </c>
+      <c r="F7" s="34">
+        <f>F5*F6</f>
+        <v>11250</v>
+      </c>
+      <c r="G7" s="34">
+        <f>G5*G6</f>
+        <v>8250</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B10" s="28" t="s">
+        <v>677</v>
+      </c>
+      <c r="C10" s="28" t="s">
+        <v>572</v>
+      </c>
+      <c r="D10" s="28" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B11">
+        <v>1003</v>
+      </c>
+      <c r="C11">
+        <f>HLOOKUP(B11,C3:G7,MATCH(B5,B3:B7,0),MATCH(B11,C3:G3,0))</f>
+        <v>45000</v>
+      </c>
+      <c r="D11">
+        <f>HLOOKUP(B11,C3:G7,MATCH(B7,B3:B7,0),MATCH(B11,C3:G3,0))</f>
+        <v>6750</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B11" xr:uid="{D0A27221-10CB-49D2-B266-F32E2FD6BE7E}">
+      <formula1>$C$3:$G$3</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>